<commit_message>
Added tools and tackles module
</commit_message>
<xml_diff>
--- a/templates/complaint_register.xlsx
+++ b/templates/complaint_register.xlsx
@@ -373,9 +373,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>1226520</xdr:colOff>
+      <xdr:colOff>1226160</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>73800</xdr:rowOff>
+      <xdr:rowOff>73440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -389,7 +389,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1730520" y="390240"/>
-          <a:ext cx="1121760" cy="826560"/>
+          <a:ext cx="1121400" cy="826200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>